<commit_message>
updated battery 1 to 3
</commit_message>
<xml_diff>
--- a/data/capacity.xlsx
+++ b/data/capacity.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\archive\github\beston-9volt-battery\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C44CF6-2F20-4D2C-B8B3-F10A2C9622BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC7D099-96C1-4291-870C-2F3CC035DED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="840" windowWidth="24825" windowHeight="14520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7710" yWindow="2085" windowWidth="19995" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="battery3" sheetId="1" r:id="rId1"/>
     <sheet name="usb_battery1" sheetId="2" r:id="rId2"/>
+    <sheet name="all" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>date</t>
   </si>
@@ -71,6 +72,69 @@
   </si>
   <si>
     <t>v_end_c</t>
+  </si>
+  <si>
+    <t>discharge mA</t>
+  </si>
+  <si>
+    <t>charge mA</t>
+  </si>
+  <si>
+    <t>discharge mAh</t>
+  </si>
+  <si>
+    <t>discharge time</t>
+  </si>
+  <si>
+    <t>discharge voltage</t>
+  </si>
+  <si>
+    <t>charge mAh</t>
+  </si>
+  <si>
+    <t>charge time</t>
+  </si>
+  <si>
+    <t>charge voltage</t>
+  </si>
+  <si>
+    <t>discharge Wh</t>
+  </si>
+  <si>
+    <t>charge Wh</t>
+  </si>
+  <si>
+    <t>battery</t>
+  </si>
+  <si>
+    <t>battery1</t>
+  </si>
+  <si>
+    <t>battery2</t>
+  </si>
+  <si>
+    <t>battery3</t>
+  </si>
+  <si>
+    <t>battery4</t>
+  </si>
+  <si>
+    <t>capacity Wh</t>
+  </si>
+  <si>
+    <t>battery5</t>
+  </si>
+  <si>
+    <t>battery6</t>
+  </si>
+  <si>
+    <t>battery7</t>
+  </si>
+  <si>
+    <t>battery8</t>
+  </si>
+  <si>
+    <t>usb_battery</t>
   </si>
 </sst>
 </file>
@@ -81,7 +145,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -93,6 +157,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -147,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -171,7 +241,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,49 +533,47 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="6.85546875" customWidth="1"/>
     <col min="7" max="8" width="7" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.28515625" customWidth="1"/>
+    <col min="11" max="11" width="7.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>9</v>
+        <v>14</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>10</v>
+        <v>17</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>18</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -877,7 +951,7 @@
       <c r="A29" s="1"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
@@ -1081,4 +1155,78 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AC39E42-60B9-4339-9FBB-23CD4F233208}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10">
+        <v>3.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>